<commit_message>
Prepare numerical study SS upload package
</commit_message>
<xml_diff>
--- a/results/simulation_results.xlsx
+++ b/results/simulation_results.xlsx
@@ -21,16 +21,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -49,21 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -437,12 +425,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>item</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
@@ -468,7 +456,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-13 12:47</t>
+          <t>2026-07-19 16:00</t>
         </is>
       </c>
     </row>
@@ -800,37 +788,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>part</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>mean_cov</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>mean_abs_dev_0.95</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>min_cov</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>max_cov</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>mean_width</t>
         </is>
@@ -902,19 +890,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.962</v>
+        <v>0.954</v>
       </c>
       <c r="D4" t="n">
-        <v>0.012</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.96</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="F4" t="n">
         <v>0.967</v>
       </c>
       <c r="G4" t="n">
-        <v>0.956</v>
+        <v>0.836</v>
       </c>
     </row>
     <row r="5">
@@ -941,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1.752</v>
+        <v>1.617</v>
       </c>
     </row>
     <row r="6">
@@ -1026,57 +1014,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>noise</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ours_coverage</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>ours_cov_mcse</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ours_width</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>cao_coverage</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>cao_width</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>width_ratio_ours_over_cao</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>h_est_mean</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>n_reps</t>
         </is>
@@ -1759,68 +1747,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>noise</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>ours_joint_coverage</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>ours_cov_mcse</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ours_width</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>h_est_mean</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>n_reps</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>bonferroni_cao_coverage</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>bonferroni_cao_width</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>width_ratio_ours_over_bonf</t>
         </is>
@@ -1833,28 +1827,33 @@
       <c r="B2" t="n">
         <v>5</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>gauss</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>0.967</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.0056</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>1.34</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0.09</v>
       </c>
-      <c r="G2" t="n">
-        <v>1000</v>
-      </c>
       <c r="H2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>1.617</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>0.829</v>
       </c>
     </row>
@@ -1863,31 +1862,36 @@
         <v>200</v>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0.96</v>
+        <v>5</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>laplace</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>0.0062</v>
+        <v>0.955</v>
       </c>
       <c r="E3" t="n">
-        <v>0.849</v>
+        <v>0.0066</v>
       </c>
       <c r="F3" t="n">
-        <v>0.07530000000000001</v>
+        <v>1.322</v>
       </c>
       <c r="G3" t="n">
-        <v>1000</v>
+        <v>0.0901</v>
       </c>
       <c r="H3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I3" t="n">
         <v>1</v>
       </c>
-      <c r="I3" t="n">
-        <v>1.775</v>
-      </c>
       <c r="J3" t="n">
-        <v>0.478</v>
+        <v>1.605</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.823</v>
       </c>
     </row>
     <row r="4">
@@ -1895,31 +1899,591 @@
         <v>200</v>
       </c>
       <c r="B4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>uniform</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.622</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.835</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>200</v>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>gauss</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.849</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.07530000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1.775</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.478</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>200</v>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>laplace</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.845</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.477</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>200</v>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>uniform</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.856</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0752</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1.782</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.48</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>200</v>
+      </c>
+      <c r="B8" t="n">
         <v>15</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>gauss</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>0.96</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E8" t="n">
         <v>0.0062</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F8" t="n">
         <v>0.68</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G8" t="n">
         <v>0.0684</v>
       </c>
-      <c r="G4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H4" t="n">
+      <c r="H8" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I8" t="n">
         <v>1</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J8" t="n">
         <v>1.863</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K8" t="n">
         <v>0.365</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>200</v>
+      </c>
+      <c r="B9" t="n">
+        <v>15</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>laplace</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.0683</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1.861</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.364</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>200</v>
+      </c>
+      <c r="B10" t="n">
+        <v>15</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>uniform</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.6830000000000001</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0682</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1.866</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.366</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>300</v>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>gauss</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.081</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.365</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>300</v>
+      </c>
+      <c r="B12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>laplace</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0063</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.0813</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1.353</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.706</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>300</v>
+      </c>
+      <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>uniform</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0.967</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.0056</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.08110000000000001</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1.364</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.712</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>300</v>
+      </c>
+      <c r="B14" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>gauss</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.0076</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.0687</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1.505</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.432</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>300</v>
+      </c>
+      <c r="B15" t="n">
+        <v>10</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>laplace</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.0074</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.648</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.0682</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1.503</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.431</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>300</v>
+      </c>
+      <c r="B16" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>uniform</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.0073</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.0683</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1.515</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.432</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>300</v>
+      </c>
+      <c r="B17" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>gauss</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.06270000000000001</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1.578</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.336</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>300</v>
+      </c>
+      <c r="B18" t="n">
+        <v>15</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>laplace</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.0076</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.0623</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>1.579</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.336</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>300</v>
+      </c>
+      <c r="B19" t="n">
+        <v>15</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>uniform</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.0071</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.0625</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1000</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1.582</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.337</v>
       </c>
     </row>
   </sheetData>
@@ -1950,57 +2514,57 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>dist</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ours_coverage</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>ours_cov_mcse</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ours_width</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>caihu_coverage</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>caihu_width</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>width_ratio_ours_over_caihu</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>h_est_mean</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>n_reps</t>
         </is>

</xml_diff>